<commit_message>
tuesday W7 populated recipes
</commit_message>
<xml_diff>
--- a/IssueTrackingTemplate.xlsx
+++ b/IssueTrackingTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Downloads\Techtorium\Level 6\Term 4\Final 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kyran\Downloads\L6 Software\Term1\Week7(RecipeApp)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF418609-59DF-421A-8EE8-8A357731DAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AA548F-8B9C-403B-92CB-D30668DD32C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5310" yWindow="-16320" windowWidth="37710" windowHeight="16440" xr2:uid="{424A518E-60D1-476D-B9C7-FC88A6A8BF20}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{424A518E-60D1-476D-B9C7-FC88A6A8BF20}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -575,21 +575,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3077EA1D-6131-4F3F-AAD9-987F0F315D03}">
   <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="43.33203125" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="43.36328125" customWidth="1"/>
+    <col min="2" max="2" width="12.36328125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="15.08984375" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.08984375" style="3" customWidth="1"/>
     <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="67.44140625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="101.6640625" customWidth="1"/>
-    <col min="10" max="10" width="29.33203125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="67.453125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="101.6328125" customWidth="1"/>
+    <col min="10" max="10" width="29.36328125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="48" customHeight="1">
+    <row r="1" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -603,7 +603,7 @@
       <c r="I1" s="17"/>
       <c r="J1" s="17"/>
     </row>
-    <row r="2" spans="1:10" s="2" customFormat="1" ht="56.4" customHeight="1">
+    <row r="2" spans="1:10" s="2" customFormat="1" ht="56.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -635,7 +635,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="1" customFormat="1" ht="250.2" customHeight="1">
+    <row r="3" spans="1:10" s="1" customFormat="1" ht="250.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="12"/>
       <c r="B3" s="11"/>
       <c r="C3" s="16"/>
@@ -647,7 +647,7 @@
       <c r="I3" s="13"/>
       <c r="J3" s="11"/>
     </row>
-    <row r="4" spans="1:10" s="1" customFormat="1" ht="237" customHeight="1">
+    <row r="4" spans="1:10" s="1" customFormat="1" ht="237" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11"/>
       <c r="B4" s="11"/>
       <c r="C4" s="16"/>
@@ -659,7 +659,7 @@
       <c r="I4" s="13"/>
       <c r="J4" s="11"/>
     </row>
-    <row r="5" spans="1:10" s="1" customFormat="1" ht="46.8" customHeight="1">
+    <row r="5" spans="1:10" s="1" customFormat="1" ht="46.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="13"/>
       <c r="B5" s="11"/>
       <c r="C5" s="12"/>
@@ -671,7 +671,7 @@
       <c r="I5" s="13"/>
       <c r="J5" s="11"/>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1">
+    <row r="6" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13"/>
       <c r="B6" s="11"/>
       <c r="C6" s="12"/>
@@ -683,7 +683,7 @@
       <c r="I6" s="13"/>
       <c r="J6" s="11"/>
     </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1">
+    <row r="7" spans="1:10" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13"/>
       <c r="B7" s="11"/>
       <c r="C7" s="12"/>
@@ -695,28 +695,28 @@
       <c r="I7" s="13"/>
       <c r="J7" s="11"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" ht="15" x14ac:dyDescent="0.4">
       <c r="A8" s="13"/>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="13"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="13"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="13"/>
       <c r="H11" s="5"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="13"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="13"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
     </row>
   </sheetData>
@@ -729,14 +729,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="df9135bc-a39e-4069-9ffb-360f93402c62" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="48ec3ddf-2ef2-4a9b-9631-68f5ec9f82f4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -955,21 +953,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="df9135bc-a39e-4069-9ffb-360f93402c62" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="48ec3ddf-2ef2-4a9b-9631-68f5ec9f82f4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B117156E-4843-4E5A-94DD-2C03D3A6E2AF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF5A31AF-7E73-46CC-A489-5A951F56E47B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="df9135bc-a39e-4069-9ffb-360f93402c62"/>
-    <ds:schemaRef ds:uri="48ec3ddf-2ef2-4a9b-9631-68f5ec9f82f4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -994,9 +991,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF5A31AF-7E73-46CC-A489-5A951F56E47B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B117156E-4843-4E5A-94DD-2C03D3A6E2AF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="df9135bc-a39e-4069-9ffb-360f93402c62"/>
+    <ds:schemaRef ds:uri="48ec3ddf-2ef2-4a9b-9631-68f5ec9f82f4"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>